<commit_message>
Initial updates for Italy
</commit_message>
<xml_diff>
--- a/input/EUROMODpolicySchedule.xlsx
+++ b/input/EUROMODpolicySchedule.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Patryk\git\SimPaths_HU\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8E657668-92E1-49D3-B746-59FD90D85C36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F04292D-C312-49E4-820D-4B845EFD099D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="993" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" tabRatio="993" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="PL" sheetId="4" r:id="rId1"/>
+    <sheet name="IT" sheetId="4" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
   <extLst>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="720" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="236" uniqueCount="62">
   <si>
     <t>Filename</t>
   </si>
@@ -82,6 +82,93 @@
   </si>
   <si>
     <t>2024</t>
+  </si>
+  <si>
+    <t>it_2011_std.txt</t>
+  </si>
+  <si>
+    <t>it_2012_std.txt</t>
+  </si>
+  <si>
+    <t>it_2013_std.txt</t>
+  </si>
+  <si>
+    <t>it_2014_std.txt</t>
+  </si>
+  <si>
+    <t>it_2015_std.txt</t>
+  </si>
+  <si>
+    <t>it_2016_std.txt</t>
+  </si>
+  <si>
+    <t>it_2017_std.txt</t>
+  </si>
+  <si>
+    <t>it_2018_std.txt</t>
+  </si>
+  <si>
+    <t>it_2019_std.txt</t>
+  </si>
+  <si>
+    <t>it_2020_std.txt</t>
+  </si>
+  <si>
+    <t>it_2021_std.txt</t>
+  </si>
+  <si>
+    <t>it_2022_std.txt</t>
+  </si>
+  <si>
+    <t>it_2023_std.txt</t>
+  </si>
+  <si>
+    <t>it_2024_std.txt</t>
+  </si>
+  <si>
+    <t>hu_2011_std.txt</t>
+  </si>
+  <si>
+    <t>hu_2012_std.txt</t>
+  </si>
+  <si>
+    <t>hu_2013_std.txt</t>
+  </si>
+  <si>
+    <t>hu_2014_std.txt</t>
+  </si>
+  <si>
+    <t>hu_2015_std.txt</t>
+  </si>
+  <si>
+    <t>hu_2016_std.txt</t>
+  </si>
+  <si>
+    <t>hu_2017_std.txt</t>
+  </si>
+  <si>
+    <t>hu_2018_std.txt</t>
+  </si>
+  <si>
+    <t>hu_2019_std.txt</t>
+  </si>
+  <si>
+    <t>hu_2020_std.txt</t>
+  </si>
+  <si>
+    <t>hu_2021_std.txt</t>
+  </si>
+  <si>
+    <t>hu_2022_std.txt</t>
+  </si>
+  <si>
+    <t>hu_2023_std.txt</t>
+  </si>
+  <si>
+    <t>hu_2024_std.txt</t>
+  </si>
+  <si>
+    <t>it_2010_std.txt</t>
   </si>
   <si>
     <t>pl_2011_std.txt</t>
@@ -476,11 +563,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{46FED923-16BB-49A3-BC38-F01A901092C1}">
-  <dimension ref="A1:D15"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:D44"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="17.85546875" collapsed="true"/>
-    <col min="2" max="1025" width="9.140625" collapsed="true"/>
+    <col min="1" max="1" customWidth="true" width="17.86328125" collapsed="true"/>
+    <col min="2" max="1025" width="9.1328125" collapsed="true"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -499,13 +586,13 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>19</v>
+        <v>33</v>
       </c>
       <c r="B2" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="C2" t="s">
-        <v>8</v>
+        <v>13</v>
       </c>
       <c r="D2" t="s">
         <v>13</v>
@@ -513,13 +600,13 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>20</v>
+        <v>34</v>
       </c>
       <c r="B3" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="C3" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="D3" t="s">
         <v>13</v>
@@ -527,13 +614,13 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>21</v>
+        <v>35</v>
       </c>
       <c r="B4" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C4" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D4" t="s">
         <v>13</v>
@@ -541,13 +628,13 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>22</v>
+        <v>36</v>
       </c>
       <c r="B5" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C5" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="D5" t="s">
         <v>13</v>
@@ -555,13 +642,13 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>23</v>
+        <v>37</v>
       </c>
       <c r="B6" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="C6" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
       <c r="D6" t="s">
         <v>13</v>
@@ -569,13 +656,13 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>24</v>
+        <v>38</v>
       </c>
       <c r="B7" t="s">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="C7" t="s">
-        <v>4</v>
+        <v>13</v>
       </c>
       <c r="D7" t="s">
         <v>13</v>
@@ -583,13 +670,13 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>25</v>
+        <v>39</v>
       </c>
       <c r="B8" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="C8" t="s">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="D8" t="s">
         <v>13</v>
@@ -597,13 +684,13 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="B9" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C9" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D9" t="s">
         <v>13</v>
@@ -611,13 +698,13 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>27</v>
+        <v>41</v>
       </c>
       <c r="B10" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="C10" t="s">
-        <v>6</v>
+        <v>13</v>
       </c>
       <c r="D10" t="s">
         <v>13</v>
@@ -625,13 +712,13 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>28</v>
+        <v>42</v>
       </c>
       <c r="B11" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="C11" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="D11" t="s">
         <v>13</v>
@@ -639,13 +726,13 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>29</v>
+        <v>43</v>
       </c>
       <c r="B12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C12" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D12" t="s">
         <v>13</v>
@@ -653,13 +740,13 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>30</v>
+        <v>44</v>
       </c>
       <c r="B13" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="C13" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D13" t="s">
         <v>13</v>
@@ -667,13 +754,13 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>31</v>
+        <v>45</v>
       </c>
       <c r="B14" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="C14" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D14" t="s">
         <v>13</v>
@@ -681,15 +768,421 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
+        <v>46</v>
+      </c>
+      <c r="B15" t="s">
+        <v>13</v>
+      </c>
+      <c r="C15" t="s">
+        <v>13</v>
+      </c>
+      <c r="D15" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>47</v>
+      </c>
+      <c r="B16" t="s">
+        <v>13</v>
+      </c>
+      <c r="C16" t="s">
+        <v>13</v>
+      </c>
+      <c r="D16" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>19</v>
+      </c>
+      <c r="B17" t="s">
+        <v>8</v>
+      </c>
+      <c r="C17" t="s">
+        <v>8</v>
+      </c>
+      <c r="D17" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>20</v>
+      </c>
+      <c r="B18" t="s">
+        <v>9</v>
+      </c>
+      <c r="C18" t="s">
+        <v>9</v>
+      </c>
+      <c r="D18" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>21</v>
+      </c>
+      <c r="B19" t="s">
+        <v>10</v>
+      </c>
+      <c r="C19" t="s">
+        <v>10</v>
+      </c>
+      <c r="D19" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>22</v>
+      </c>
+      <c r="B20" t="s">
+        <v>11</v>
+      </c>
+      <c r="C20" t="s">
+        <v>11</v>
+      </c>
+      <c r="D20" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s">
+        <v>23</v>
+      </c>
+      <c r="B21" t="s">
+        <v>3</v>
+      </c>
+      <c r="C21" t="s">
+        <v>3</v>
+      </c>
+      <c r="D21" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s">
+        <v>24</v>
+      </c>
+      <c r="B22" t="s">
+        <v>4</v>
+      </c>
+      <c r="C22" t="s">
+        <v>4</v>
+      </c>
+      <c r="D22" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s">
+        <v>25</v>
+      </c>
+      <c r="B23" t="s">
+        <v>5</v>
+      </c>
+      <c r="C23" t="s">
+        <v>5</v>
+      </c>
+      <c r="D23" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="s">
+        <v>26</v>
+      </c>
+      <c r="B24" t="s">
+        <v>12</v>
+      </c>
+      <c r="C24" t="s">
+        <v>12</v>
+      </c>
+      <c r="D24" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s">
+        <v>27</v>
+      </c>
+      <c r="B25" t="s">
+        <v>6</v>
+      </c>
+      <c r="C25" t="s">
+        <v>6</v>
+      </c>
+      <c r="D25" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="s">
+        <v>28</v>
+      </c>
+      <c r="B26" t="s">
+        <v>7</v>
+      </c>
+      <c r="C26" t="s">
+        <v>7</v>
+      </c>
+      <c r="D26" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="s">
+        <v>29</v>
+      </c>
+      <c r="B27" t="s">
+        <v>14</v>
+      </c>
+      <c r="C27" t="s">
+        <v>14</v>
+      </c>
+      <c r="D27" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="s">
+        <v>30</v>
+      </c>
+      <c r="B28" t="s">
+        <v>16</v>
+      </c>
+      <c r="C28" t="s">
+        <v>16</v>
+      </c>
+      <c r="D28" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="s">
+        <v>31</v>
+      </c>
+      <c r="B29" t="s">
+        <v>17</v>
+      </c>
+      <c r="C29" t="s">
+        <v>17</v>
+      </c>
+      <c r="D29" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="s">
         <v>32</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B30" t="s">
         <v>18</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C30" t="s">
         <v>18</v>
       </c>
-      <c r="D15" t="s">
+      <c r="D30" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="s">
+        <v>48</v>
+      </c>
+      <c r="B31" t="s">
+        <v>13</v>
+      </c>
+      <c r="C31" t="s">
+        <v>13</v>
+      </c>
+      <c r="D31" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="s">
+        <v>49</v>
+      </c>
+      <c r="B32" t="s">
+        <v>13</v>
+      </c>
+      <c r="C32" t="s">
+        <v>13</v>
+      </c>
+      <c r="D32" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="s">
+        <v>50</v>
+      </c>
+      <c r="B33" t="s">
+        <v>13</v>
+      </c>
+      <c r="C33" t="s">
+        <v>13</v>
+      </c>
+      <c r="D33" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="s">
+        <v>51</v>
+      </c>
+      <c r="B34" t="s">
+        <v>13</v>
+      </c>
+      <c r="C34" t="s">
+        <v>13</v>
+      </c>
+      <c r="D34" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="s">
+        <v>52</v>
+      </c>
+      <c r="B35" t="s">
+        <v>13</v>
+      </c>
+      <c r="C35" t="s">
+        <v>13</v>
+      </c>
+      <c r="D35" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="s">
+        <v>53</v>
+      </c>
+      <c r="B36" t="s">
+        <v>13</v>
+      </c>
+      <c r="C36" t="s">
+        <v>13</v>
+      </c>
+      <c r="D36" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="s">
+        <v>54</v>
+      </c>
+      <c r="B37" t="s">
+        <v>13</v>
+      </c>
+      <c r="C37" t="s">
+        <v>13</v>
+      </c>
+      <c r="D37" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="s">
+        <v>55</v>
+      </c>
+      <c r="B38" t="s">
+        <v>13</v>
+      </c>
+      <c r="C38" t="s">
+        <v>13</v>
+      </c>
+      <c r="D38" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="s">
+        <v>56</v>
+      </c>
+      <c r="B39" t="s">
+        <v>13</v>
+      </c>
+      <c r="C39" t="s">
+        <v>13</v>
+      </c>
+      <c r="D39" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="s">
+        <v>57</v>
+      </c>
+      <c r="B40" t="s">
+        <v>13</v>
+      </c>
+      <c r="C40" t="s">
+        <v>13</v>
+      </c>
+      <c r="D40" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="s">
+        <v>58</v>
+      </c>
+      <c r="B41" t="s">
+        <v>13</v>
+      </c>
+      <c r="C41" t="s">
+        <v>13</v>
+      </c>
+      <c r="D41" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="s">
+        <v>59</v>
+      </c>
+      <c r="B42" t="s">
+        <v>13</v>
+      </c>
+      <c r="C42" t="s">
+        <v>13</v>
+      </c>
+      <c r="D42" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="s">
+        <v>60</v>
+      </c>
+      <c r="B43" t="s">
+        <v>13</v>
+      </c>
+      <c r="C43" t="s">
+        <v>13</v>
+      </c>
+      <c r="D43" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="s">
+        <v>61</v>
+      </c>
+      <c r="B44" t="s">
+        <v>13</v>
+      </c>
+      <c r="C44" t="s">
+        <v>13</v>
+      </c>
+      <c r="D44" t="s">
         <v>13</v>
       </c>
     </row>

</xml_diff>

<commit_message>
add lifetime income measure to person object
</commit_message>
<xml_diff>
--- a/input/EUROMODpolicySchedule.xlsx
+++ b/input/EUROMODpolicySchedule.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="45">
   <si>
     <t>Filename</t>
   </si>
@@ -631,7 +631,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5CC6207-DD24-427A-A7C5-E1B68985A6D0}">
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" customWidth="true" width="17.85546875" collapsed="true"/>
@@ -680,146 +680,6 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="s">
-        <v>24</v>
-      </c>
-      <c r="B4" t="s">
-        <v>8</v>
-      </c>
-      <c r="C4" t="s">
-        <v>8</v>
-      </c>
-      <c r="D4" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="s">
-        <v>25</v>
-      </c>
-      <c r="B5" t="s">
-        <v>28</v>
-      </c>
-      <c r="C5" t="s">
-        <v>28</v>
-      </c>
-      <c r="D5" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="s">
-        <v>29</v>
-      </c>
-      <c r="B6" t="s">
-        <v>30</v>
-      </c>
-      <c r="C6" t="s">
-        <v>30</v>
-      </c>
-      <c r="D6" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="s">
-        <v>31</v>
-      </c>
-      <c r="B7" t="s">
-        <v>32</v>
-      </c>
-      <c r="C7" t="s">
-        <v>32</v>
-      </c>
-      <c r="D7" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="s">
-        <v>33</v>
-      </c>
-      <c r="B8" t="s">
-        <v>34</v>
-      </c>
-      <c r="C8" t="s">
-        <v>34</v>
-      </c>
-      <c r="D8" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="s">
-        <v>35</v>
-      </c>
-      <c r="B9" t="s">
-        <v>36</v>
-      </c>
-      <c r="C9" t="s">
-        <v>36</v>
-      </c>
-      <c r="D9" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="s">
-        <v>37</v>
-      </c>
-      <c r="B10" t="s">
-        <v>38</v>
-      </c>
-      <c r="C10" t="s">
-        <v>38</v>
-      </c>
-      <c r="D10" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="s">
-        <v>39</v>
-      </c>
-      <c r="B11" t="s">
-        <v>40</v>
-      </c>
-      <c r="C11" t="s">
-        <v>40</v>
-      </c>
-      <c r="D11" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="s">
-        <v>41</v>
-      </c>
-      <c r="B12" t="s">
-        <v>42</v>
-      </c>
-      <c r="C12" t="s">
-        <v>42</v>
-      </c>
-      <c r="D12" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="s">
-        <v>43</v>
-      </c>
-      <c r="B13" t="s">
-        <v>44</v>
-      </c>
-      <c r="C13" t="s">
-        <v>44</v>
-      </c>
-      <c r="D13" t="s">
-        <v>12</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.51180555555555496" footer="0.51180555555555496"/>
   <pageSetup paperSize="0" scale="0" firstPageNumber="0" orientation="portrait" usePrinterDefaults="0" horizontalDpi="0" verticalDpi="0" copies="0"/>

</xml_diff>

<commit_message>
update output files for integration test
</commit_message>
<xml_diff>
--- a/input/EUROMODpolicySchedule.xlsx
+++ b/input/EUROMODpolicySchedule.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24326"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent>
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MyFiles\99 DEV ENV\JAS-MINE\SimPaths\input\EUROMODoutput\current\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Patryk\git\labsim_Italy\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3402BA8E-92CD-40B8-B77E-691FC16035DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95F0610D-9867-49D9-9F5B-A4E2213BB68C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="993" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="20400" tabRatio="993" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="IT" sheetId="1" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="329" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17312" uniqueCount="61">
   <si>
     <t>Filename</t>
   </si>
@@ -151,6 +151,54 @@
     <t>2024</t>
   </si>
   <si>
+    <t>uk_2021_10_std.txt</t>
+  </si>
+  <si>
+    <t>uk_2022_10_std.txt</t>
+  </si>
+  <si>
+    <t>uk_2023_10_std.txt</t>
+  </si>
+  <si>
+    <t>uk_2024_10_std.txt</t>
+  </si>
+  <si>
+    <t>uk_2010_std.txt</t>
+  </si>
+  <si>
+    <t>hscl_uk_2017_std.txt</t>
+  </si>
+  <si>
+    <t>hscl_uk_2018_std.txt</t>
+  </si>
+  <si>
+    <t>hscl_uk_2019_std.txt</t>
+  </si>
+  <si>
+    <t>hscl_uk_2020_std.txt</t>
+  </si>
+  <si>
+    <t>hscl_uk_2021_std.txt</t>
+  </si>
+  <si>
+    <t>hscl_uk_2022_std.txt</t>
+  </si>
+  <si>
+    <t>hscl_uk_2023_std.txt</t>
+  </si>
+  <si>
+    <t>hscl_uk_2024_std.txt</t>
+  </si>
+  <si>
+    <t>uk_2022_nohscl_std.txt</t>
+  </si>
+  <si>
+    <t>uk_2023_nohscl_std.txt</t>
+  </si>
+  <si>
+    <t>uk_2024_nohscl_std.txt</t>
+  </si>
+  <si>
     <t>uk_2025_std.txt</t>
   </si>
   <si>
@@ -161,24 +209,6 @@
   </si>
   <si>
     <t>2026</t>
-  </si>
-  <si>
-    <t>uk_2027_std.txt</t>
-  </si>
-  <si>
-    <t>2027</t>
-  </si>
-  <si>
-    <t>uk_2028_std.txt</t>
-  </si>
-  <si>
-    <t>2028</t>
-  </si>
-  <si>
-    <t>uk_2029_std.txt</t>
-  </si>
-  <si>
-    <t>2029</t>
   </si>
 </sst>
 </file>
@@ -235,9 +265,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -275,7 +305,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -381,7 +411,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -523,7 +553,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -535,7 +565,8 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" customWidth="true" width="17.85546875" collapsed="true"/>
-    <col min="2" max="3" customWidth="true" width="14.0" collapsed="true"/>
+    <col min="2" max="2" customWidth="true" width="14.0" collapsed="true"/>
+    <col min="3" max="3" customWidth="true" width="14.0" collapsed="true"/>
     <col min="4" max="1026" width="8.7109375" collapsed="true"/>
   </cols>
   <sheetData>
@@ -649,7 +680,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5CC6207-DD24-427A-A7C5-E1B68985A6D0}">
-  <dimension ref="A1:D20"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" customWidth="true" width="17.85546875" collapsed="true"/>
@@ -868,13 +899,13 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>41</v>
+        <v>57</v>
       </c>
       <c r="B16" t="s">
-        <v>42</v>
+        <v>58</v>
       </c>
       <c r="C16" t="s">
-        <v>42</v>
+        <v>58</v>
       </c>
       <c r="D16" t="s">
         <v>19</v>
@@ -882,57 +913,15 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>43</v>
+        <v>59</v>
       </c>
       <c r="B17" t="s">
-        <v>44</v>
+        <v>60</v>
       </c>
       <c r="C17" t="s">
-        <v>44</v>
+        <v>60</v>
       </c>
       <c r="D17" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="s">
-        <v>45</v>
-      </c>
-      <c r="B18" t="s">
-        <v>46</v>
-      </c>
-      <c r="C18" t="s">
-        <v>46</v>
-      </c>
-      <c r="D18" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="s">
-        <v>47</v>
-      </c>
-      <c r="B19" t="s">
-        <v>48</v>
-      </c>
-      <c r="C19" t="s">
-        <v>48</v>
-      </c>
-      <c r="D19" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="s">
-        <v>49</v>
-      </c>
-      <c r="B20" t="s">
-        <v>50</v>
-      </c>
-      <c r="C20" t="s">
-        <v>50</v>
-      </c>
-      <c r="D20" t="s">
         <v>19</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Local changes before switching to develop
</commit_message>
<xml_diff>
--- a/input/EUROMODpolicySchedule.xlsx
+++ b/input/EUROMODpolicySchedule.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17312" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17380" uniqueCount="61">
   <si>
     <t>Filename</t>
   </si>
@@ -703,13 +703,13 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="B2" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="C2" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="D2" t="s">
         <v>19</v>
@@ -717,13 +717,13 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="B3" t="s">
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="C3" t="s">
-        <v>12</v>
+        <v>36</v>
       </c>
       <c r="D3" t="s">
         <v>19</v>
@@ -731,13 +731,13 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>27</v>
+        <v>37</v>
       </c>
       <c r="B4" t="s">
-        <v>13</v>
+        <v>38</v>
       </c>
       <c r="C4" t="s">
-        <v>13</v>
+        <v>38</v>
       </c>
       <c r="D4" t="s">
         <v>19</v>
@@ -745,13 +745,13 @@
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="B5" t="s">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="C5" t="s">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="D5" t="s">
         <v>19</v>
@@ -759,13 +759,13 @@
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>22</v>
+        <v>32</v>
       </c>
       <c r="B6" t="s">
-        <v>4</v>
+        <v>33</v>
       </c>
       <c r="C6" t="s">
-        <v>4</v>
+        <v>33</v>
       </c>
       <c r="D6" t="s">
         <v>19</v>
@@ -773,13 +773,13 @@
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="B7" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C7" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D7" t="s">
         <v>19</v>
@@ -787,13 +787,13 @@
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="B8" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C8" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="D8" t="s">
         <v>19</v>
@@ -801,13 +801,13 @@
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B9" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="C9" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D9" t="s">
         <v>19</v>
@@ -815,13 +815,13 @@
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>24</v>
+        <v>57</v>
       </c>
       <c r="B10" t="s">
-        <v>8</v>
+        <v>58</v>
       </c>
       <c r="C10" t="s">
-        <v>8</v>
+        <v>58</v>
       </c>
       <c r="D10" t="s">
         <v>19</v>
@@ -829,13 +829,13 @@
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="B11" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C11" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D11" t="s">
         <v>19</v>
@@ -843,13 +843,13 @@
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="B12" t="s">
-        <v>33</v>
+        <v>12</v>
       </c>
       <c r="C12" t="s">
-        <v>33</v>
+        <v>12</v>
       </c>
       <c r="D12" t="s">
         <v>19</v>
@@ -857,13 +857,13 @@
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="B13" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="C13" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="D13" t="s">
         <v>19</v>
@@ -871,13 +871,13 @@
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>37</v>
+        <v>24</v>
       </c>
       <c r="B14" t="s">
-        <v>38</v>
+        <v>8</v>
       </c>
       <c r="C14" t="s">
-        <v>38</v>
+        <v>8</v>
       </c>
       <c r="D14" t="s">
         <v>19</v>
@@ -885,13 +885,13 @@
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>39</v>
+        <v>59</v>
       </c>
       <c r="B15" t="s">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="C15" t="s">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="D15" t="s">
         <v>19</v>
@@ -899,13 +899,13 @@
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>57</v>
+        <v>30</v>
       </c>
       <c r="B16" t="s">
-        <v>58</v>
+        <v>15</v>
       </c>
       <c r="C16" t="s">
-        <v>58</v>
+        <v>15</v>
       </c>
       <c r="D16" t="s">
         <v>19</v>
@@ -913,13 +913,13 @@
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>59</v>
+        <v>25</v>
       </c>
       <c r="B17" t="s">
-        <v>60</v>
+        <v>11</v>
       </c>
       <c r="C17" t="s">
-        <v>60</v>
+        <v>11</v>
       </c>
       <c r="D17" t="s">
         <v>19</v>

</xml_diff>

<commit_message>
Added more diagnostic flags to investigate the pattern related to low matched ratios
</commit_message>
<xml_diff>
--- a/input/EUROMODpolicySchedule.xlsx
+++ b/input/EUROMODpolicySchedule.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17468" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17604" uniqueCount="61">
   <si>
     <t>Filename</t>
   </si>
@@ -680,7 +680,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5CC6207-DD24-427A-A7C5-E1B68985A6D0}">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" customWidth="true" width="17.85546875" collapsed="true"/>
@@ -703,13 +703,13 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="B2" t="s">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="C2" t="s">
-        <v>4</v>
+        <v>19</v>
       </c>
       <c r="D2" t="s">
         <v>19</v>
@@ -717,15 +717,211 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
+        <v>26</v>
+      </c>
+      <c r="B3" t="s">
+        <v>19</v>
+      </c>
+      <c r="C3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C5" t="s">
+        <v>19</v>
+      </c>
+      <c r="D5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" t="s">
+        <v>4</v>
+      </c>
+      <c r="D6" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" t="s">
+        <v>19</v>
+      </c>
+      <c r="D7" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" t="s">
+        <v>19</v>
+      </c>
+      <c r="C8" t="s">
+        <v>19</v>
+      </c>
+      <c r="D8" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>30</v>
+      </c>
+      <c r="B9" t="s">
+        <v>19</v>
+      </c>
+      <c r="C9" t="s">
+        <v>19</v>
+      </c>
+      <c r="D9" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>24</v>
+      </c>
+      <c r="B10" t="s">
+        <v>19</v>
+      </c>
+      <c r="C10" t="s">
+        <v>19</v>
+      </c>
+      <c r="D10" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>31</v>
+      </c>
+      <c r="B11" t="s">
+        <v>19</v>
+      </c>
+      <c r="C11" t="s">
+        <v>19</v>
+      </c>
+      <c r="D11" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>32</v>
+      </c>
+      <c r="B12" t="s">
+        <v>19</v>
+      </c>
+      <c r="C12" t="s">
+        <v>19</v>
+      </c>
+      <c r="D12" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>35</v>
+      </c>
+      <c r="B13" t="s">
+        <v>19</v>
+      </c>
+      <c r="C13" t="s">
+        <v>19</v>
+      </c>
+      <c r="D13" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>37</v>
+      </c>
+      <c r="B14" t="s">
+        <v>19</v>
+      </c>
+      <c r="C14" t="s">
+        <v>19</v>
+      </c>
+      <c r="D14" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>39</v>
+      </c>
+      <c r="B15" t="s">
+        <v>19</v>
+      </c>
+      <c r="C15" t="s">
+        <v>19</v>
+      </c>
+      <c r="D15" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
         <v>57</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B16" t="s">
         <v>58</v>
       </c>
-      <c r="C3" t="s">
+      <c r="C16" t="s">
         <v>58</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D16" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>59</v>
+      </c>
+      <c r="B17" t="s">
+        <v>19</v>
+      </c>
+      <c r="C17" t="s">
+        <v>19</v>
+      </c>
+      <c r="D17" t="s">
         <v>19</v>
       </c>
     </row>

</xml_diff>

<commit_message>
last batch of update, integration test passed
</commit_message>
<xml_diff>
--- a/input/EUROMODpolicySchedule.xlsx
+++ b/input/EUROMODpolicySchedule.xlsx
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17480" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17312" uniqueCount="61">
   <si>
     <t>Filename</t>
   </si>
@@ -209,12 +209,6 @@
   </si>
   <si>
     <t>2026</t>
-  </si>
-  <si>
-    <t>uk_2030_std.txt</t>
-  </si>
-  <si>
-    <t>2030</t>
   </si>
 </sst>
 </file>
@@ -686,7 +680,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5CC6207-DD24-427A-A7C5-E1B68985A6D0}">
-  <dimension ref="A1:D3"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" customWidth="true" width="17.85546875" collapsed="true"/>
@@ -709,13 +703,13 @@
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="B2" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="C2" t="s">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="D2" t="s">
         <v>19</v>
@@ -723,15 +717,211 @@
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>61</v>
+        <v>26</v>
       </c>
       <c r="B3" t="s">
-        <v>62</v>
+        <v>12</v>
       </c>
       <c r="C3" t="s">
-        <v>62</v>
+        <v>12</v>
       </c>
       <c r="D3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
+        <v>13</v>
+      </c>
+      <c r="D4" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>28</v>
+      </c>
+      <c r="B5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" t="s">
+        <v>4</v>
+      </c>
+      <c r="D6" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" t="s">
+        <v>5</v>
+      </c>
+      <c r="D7" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>29</v>
+      </c>
+      <c r="B8" t="s">
+        <v>7</v>
+      </c>
+      <c r="C8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D8" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>30</v>
+      </c>
+      <c r="B9" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" t="s">
+        <v>15</v>
+      </c>
+      <c r="D9" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s">
+        <v>24</v>
+      </c>
+      <c r="B10" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" t="s">
+        <v>8</v>
+      </c>
+      <c r="D10" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s">
+        <v>31</v>
+      </c>
+      <c r="B11" t="s">
+        <v>10</v>
+      </c>
+      <c r="C11" t="s">
+        <v>10</v>
+      </c>
+      <c r="D11" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s">
+        <v>32</v>
+      </c>
+      <c r="B12" t="s">
+        <v>33</v>
+      </c>
+      <c r="C12" t="s">
+        <v>33</v>
+      </c>
+      <c r="D12" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s">
+        <v>35</v>
+      </c>
+      <c r="B13" t="s">
+        <v>36</v>
+      </c>
+      <c r="C13" t="s">
+        <v>36</v>
+      </c>
+      <c r="D13" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s">
+        <v>37</v>
+      </c>
+      <c r="B14" t="s">
+        <v>38</v>
+      </c>
+      <c r="C14" t="s">
+        <v>38</v>
+      </c>
+      <c r="D14" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s">
+        <v>39</v>
+      </c>
+      <c r="B15" t="s">
+        <v>40</v>
+      </c>
+      <c r="C15" t="s">
+        <v>40</v>
+      </c>
+      <c r="D15" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>57</v>
+      </c>
+      <c r="B16" t="s">
+        <v>58</v>
+      </c>
+      <c r="C16" t="s">
+        <v>58</v>
+      </c>
+      <c r="D16" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>59</v>
+      </c>
+      <c r="B17" t="s">
+        <v>60</v>
+      </c>
+      <c r="C17" t="s">
+        <v>60</v>
+      </c>
+      <c r="D17" t="s">
         <v>19</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Remove IT in input Excel data files
These are "data cleaning" updates (no code changes).
</commit_message>
<xml_diff>
--- a/input/EUROMODpolicySchedule.xlsx
+++ b/input/EUROMODpolicySchedule.xlsx
@@ -1,20 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
   <workbookPr defaultThemeVersion="166925"/>
-  <mc:AlternateContent>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Patryk\git\labsim_Italy\input\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/Sonnewald/GitHub/SimPaths/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95F0610D-9867-49D9-9F5B-A4E2213BB68C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{317F52AE-B0D0-104B-BBEA-5D1B3B26490E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="20400" tabRatio="993" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="38400" windowHeight="19580" tabRatio="993" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="IT" sheetId="1" r:id="rId1"/>
-    <sheet name="UK" sheetId="2" r:id="rId2"/>
+    <sheet name="UK" sheetId="2" r:id="rId1"/>
   </sheets>
   <calcPr calcId="0"/>
   <extLst>
@@ -26,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17528" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="9">
   <si>
     <t>Filename</t>
   </si>
@@ -37,178 +36,16 @@
     <t>Description</t>
   </si>
   <si>
-    <t>it_2016_std.txt</t>
-  </si>
-  <si>
     <t>2015</t>
   </si>
   <si>
-    <t>2016</t>
-  </si>
-  <si>
-    <t>it_2015_std.txt</t>
-  </si>
-  <si>
-    <t>2017</t>
-  </si>
-  <si>
-    <t>2019</t>
-  </si>
-  <si>
-    <t>it_2020_web_std.txt</t>
-  </si>
-  <si>
-    <t>2020</t>
-  </si>
-  <si>
-    <t>2011</t>
-  </si>
-  <si>
-    <t>2012</t>
-  </si>
-  <si>
-    <t>2013</t>
-  </si>
-  <si>
-    <t>2014</t>
-  </si>
-  <si>
-    <t>2018</t>
-  </si>
-  <si>
-    <t>Policy for 2015</t>
-  </si>
-  <si>
-    <t>Policy for 2016</t>
-  </si>
-  <si>
-    <t>Policy for 2020 onwards</t>
-  </si>
-  <si>
     <t/>
   </si>
   <si>
-    <t>it_2020_web_std_v2.txt</t>
-  </si>
-  <si>
-    <t>uk_2015_e7_std.txt</t>
-  </si>
-  <si>
     <t>uk_2015_std.txt</t>
   </si>
   <si>
-    <t>uk_2016_std.txt</t>
-  </si>
-  <si>
-    <t>uk_2019_std.txt</t>
-  </si>
-  <si>
-    <t>uk_2011_std.txt</t>
-  </si>
-  <si>
-    <t>uk_2012_std.txt</t>
-  </si>
-  <si>
-    <t>uk_2013_std.txt</t>
-  </si>
-  <si>
-    <t>uk_2014_std.txt</t>
-  </si>
-  <si>
-    <t>uk_2017_std.txt</t>
-  </si>
-  <si>
-    <t>uk_2018_std.txt</t>
-  </si>
-  <si>
-    <t>uk_2020_std.txt</t>
-  </si>
-  <si>
-    <t>uk_2021_std.txt</t>
-  </si>
-  <si>
-    <t>2021</t>
-  </si>
-  <si>
     <t>Policy_System_Year</t>
-  </si>
-  <si>
-    <t>uk_2022_std.txt</t>
-  </si>
-  <si>
-    <t>2022</t>
-  </si>
-  <si>
-    <t>uk_2023_std.txt</t>
-  </si>
-  <si>
-    <t>2023</t>
-  </si>
-  <si>
-    <t>uk_2024_std.txt</t>
-  </si>
-  <si>
-    <t>2024</t>
-  </si>
-  <si>
-    <t>uk_2021_10_std.txt</t>
-  </si>
-  <si>
-    <t>uk_2022_10_std.txt</t>
-  </si>
-  <si>
-    <t>uk_2023_10_std.txt</t>
-  </si>
-  <si>
-    <t>uk_2024_10_std.txt</t>
-  </si>
-  <si>
-    <t>uk_2010_std.txt</t>
-  </si>
-  <si>
-    <t>hscl_uk_2017_std.txt</t>
-  </si>
-  <si>
-    <t>hscl_uk_2018_std.txt</t>
-  </si>
-  <si>
-    <t>hscl_uk_2019_std.txt</t>
-  </si>
-  <si>
-    <t>hscl_uk_2020_std.txt</t>
-  </si>
-  <si>
-    <t>hscl_uk_2021_std.txt</t>
-  </si>
-  <si>
-    <t>hscl_uk_2022_std.txt</t>
-  </si>
-  <si>
-    <t>hscl_uk_2023_std.txt</t>
-  </si>
-  <si>
-    <t>hscl_uk_2024_std.txt</t>
-  </si>
-  <si>
-    <t>uk_2022_nohscl_std.txt</t>
-  </si>
-  <si>
-    <t>uk_2023_nohscl_std.txt</t>
-  </si>
-  <si>
-    <t>uk_2024_nohscl_std.txt</t>
-  </si>
-  <si>
-    <t>uk_2025_std.txt</t>
-  </si>
-  <si>
-    <t>2025</t>
-  </si>
-  <si>
-    <t>uk_2026_std.txt</t>
-  </si>
-  <si>
-    <t>2026</t>
   </si>
   <si>
     <t>uk_2030_std.txt</t>
@@ -221,7 +58,6 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="0"/>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -271,9 +107,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -311,7 +147,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -417,7 +253,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -559,24 +395,22 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5CC6207-DD24-427A-A7C5-E1B68985A6D0}">
+  <dimension ref="A1:AMK3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" customWidth="true" width="17.85546875" collapsed="true"/>
-    <col min="2" max="2" customWidth="true" width="14.0" collapsed="true"/>
-    <col min="3" max="3" customWidth="true" width="14.0" collapsed="true"/>
-    <col min="4" max="1026" width="8.7109375" collapsed="true"/>
+    <col min="1" max="1" width="17.83203125" customWidth="1" collapsed="1"/>
+    <col min="2" max="1025" width="9.1640625" collapsed="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -584,155 +418,38 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>34</v>
+        <v>6</v>
       </c>
       <c r="D1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" t="s">
         <v>4</v>
       </c>
-      <c r="D2" t="s">
-        <v>16</v>
-      </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="B3" t="s">
-        <v>5</v>
+        <v>8</v>
+      </c>
+      <c r="C3" t="s">
+        <v>8</v>
       </c>
       <c r="D3" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>9</v>
-      </c>
-      <c r="B4" t="s">
-        <v>10</v>
-      </c>
-      <c r="D4" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>20</v>
-      </c>
-      <c r="B5" t="s">
-        <v>19</v>
-      </c>
-      <c r="D5" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>21</v>
-      </c>
-      <c r="B6" t="s">
-        <v>19</v>
-      </c>
-      <c r="D6" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>22</v>
-      </c>
-      <c r="B7" t="s">
-        <v>19</v>
-      </c>
-      <c r="D7" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>23</v>
-      </c>
-      <c r="B8" t="s">
-        <v>19</v>
-      </c>
-      <c r="D8" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>24</v>
-      </c>
-      <c r="B9" t="s">
-        <v>19</v>
-      </c>
-      <c r="D9" t="s">
-        <v>19</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.51180555555555496" footer="0.51180555555555496"/>
-  <pageSetup paperSize="0" scale="0" firstPageNumber="0" orientation="portrait" usePrinterDefaults="0" horizontalDpi="0" verticalDpi="0" copies="0"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C5CC6207-DD24-427A-A7C5-E1B68985A6D0}">
-  <dimension ref="A1:D3"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" customWidth="true" width="17.85546875" collapsed="true"/>
-    <col min="2" max="1025" width="9.140625" collapsed="true"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
-        <v>34</v>
-      </c>
-      <c r="D1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="s">
-        <v>22</v>
-      </c>
-      <c r="B2" t="s">
         <v>4</v>
-      </c>
-      <c r="C2" t="s">
-        <v>4</v>
-      </c>
-      <c r="D2" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="s">
-        <v>61</v>
-      </c>
-      <c r="B3" t="s">
-        <v>62</v>
-      </c>
-      <c r="C3" t="s">
-        <v>62</v>
-      </c>
-      <c r="D3" t="s">
-        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>